<commit_message>
Stabilization pass for PAR sheet import/export
Makes export atomic (full preflight before any write; error means the
output file is neither created nor modified), forbids lossy export
when reelStripGeneration/symbolWeights are present even alongside a
literal reelStrips, and tightens ReelStrips/Paylines header parsing to
the exact "Reel 1".."Reel N" names (unknown/duplicate/missing columns
now get their own diagnostics instead of silently becoming reel data).

Provenance is now structured on ParSheetImportResult and verified
against a canonically-hashed reconstruction of the imported blueprint,
so a hand-edited workbook is reported as a hash mismatch instead of
silently accepted.
</commit_message>
<xml_diff>
--- a/examples/parsheets/starter.par.xlsx
+++ b/examples/parsheets/starter.par.xlsx
@@ -115,7 +115,7 @@
     <t>Exported At</t>
   </si>
   <si>
-    <t>2026-07-14T10:24:17.255Z</t>
+    <t>2026-07-14T12:26:28.620Z</t>
   </si>
   <si>
     <t>Source</t>
@@ -127,7 +127,7 @@
     <t>Blueprint Hash</t>
   </si>
   <si>
-    <t>sha256:6b44e45bafde479a8f2f193184e32e9d078242812788658c3a447b55600b1fa3</t>
+    <t>sha256:c86e2b261d9091e555b17b84a2eca35cf47fdd52b2d5cb963a31dfcf08362c32</t>
   </si>
 </sst>
 </file>

</xml_diff>